<commit_message>
feat(anomaly-arbitration): G13-P3-B6 verify exports and visual review
</commit_message>
<xml_diff>
--- a/config/anomaly-arbitration-generated/templates/AnomalyArbitration.xlsx
+++ b/config/anomaly-arbitration-generated/templates/AnomalyArbitration.xlsx
@@ -35,7 +35,7 @@
     <t>@table</t>
   </si>
   <si>
-    <t>AAProfiles</t>
+    <t>ArbProfiles</t>
   </si>
   <si>
     <t>@mode</t>
@@ -59,7 +59,7 @@
     <t>@schema</t>
   </si>
   <si>
-    <t>5d70693774e187ee</t>
+    <t>8e41c1906287fe2d</t>
   </si>
   <si>
     <t>#name</t>
@@ -122,16 +122,16 @@
     <t>string</t>
   </si>
   <si>
-    <t>enum&lt;AAOwnership&gt;</t>
-  </si>
-  <si>
-    <t>enum&lt;AACoverageState&gt;</t>
-  </si>
-  <si>
-    <t>enum&lt;AAEvidenceQuality&gt;</t>
-  </si>
-  <si>
-    <t>enum&lt;AAMechanismQuality&gt;</t>
+    <t>enum&lt;ArbOwnership&gt;</t>
+  </si>
+  <si>
+    <t>enum&lt;ArbCoverageState&gt;</t>
+  </si>
+  <si>
+    <t>enum&lt;ArbEvidenceQuality&gt;</t>
+  </si>
+  <si>
+    <t>enum&lt;ArbMechanismQuality&gt;</t>
   </si>
   <si>
     <t>list&lt;string&gt;</t>
@@ -176,10 +176,10 @@
     <t>#desc</t>
   </si>
   <si>
-    <t>AAPeriods</t>
-  </si>
-  <si>
-    <t>223cc75d080562d7</t>
+    <t>ArbPeriods</t>
+  </si>
+  <si>
+    <t>de07eb78dcf1943b</t>
   </si>
   <si>
     <t>profile_id</t>
@@ -188,16 +188,16 @@
     <t>source_group_id</t>
   </si>
   <si>
-    <t>ref&lt;AAProfiles.id&gt;</t>
+    <t>ref&lt;ArbProfiles.id&gt;</t>
   </si>
   <si>
     <t>length=1..64</t>
   </si>
   <si>
-    <t>AAStages</t>
-  </si>
-  <si>
-    <t>6f4c5caac5fbb95b</t>
+    <t>ArbStages</t>
+  </si>
+  <si>
+    <t>8ffccf69075880d3</t>
   </si>
   <si>
     <t>period_id</t>
@@ -215,28 +215,28 @@
     <t>difficulty</t>
   </si>
   <si>
-    <t>ref&lt;AAPeriods.id&gt;</t>
-  </si>
-  <si>
-    <t>enum&lt;AAStageKind&gt;</t>
-  </si>
-  <si>
-    <t>enum&lt;AADifficulty&gt;</t>
+    <t>ref&lt;ArbPeriods.id&gt;</t>
+  </si>
+  <si>
+    <t>enum&lt;ArbStageKind&gt;</t>
+  </si>
+  <si>
+    <t>enum&lt;ArbDifficulty&gt;</t>
   </si>
   <si>
     <t>range=1..5</t>
   </si>
   <si>
-    <t>AATerminalOutcomes</t>
-  </si>
-  <si>
-    <t>5bffe88df6082748</t>
-  </si>
-  <si>
-    <t>AAParticipantPolicies</t>
-  </si>
-  <si>
-    <t>e677d36fd26625cb</t>
+    <t>ArbTerminalOutcomes</t>
+  </si>
+  <si>
+    <t>f9d1cb1fa03f3370</t>
+  </si>
+  <si>
+    <t>ArbParticipantPolicies</t>
+  </si>
+  <si>
+    <t>24185a86735a18a9</t>
   </si>
   <si>
     <t>row_order</t>
@@ -245,10 +245,10 @@
     <t>range=1..100</t>
   </si>
   <si>
-    <t>AATeamSlots</t>
-  </si>
-  <si>
-    <t>5cfa3d3cd764b78f</t>
+    <t>ArbTeamSlots</t>
+  </si>
+  <si>
+    <t>5f629bd6046c6c98</t>
   </si>
   <si>
     <t>stage_id</t>
@@ -257,43 +257,43 @@
     <t>slot_order</t>
   </si>
   <si>
-    <t>ref&lt;AAStages.id&gt;</t>
+    <t>ref&lt;ArbStages.id&gt;</t>
   </si>
   <si>
     <t>range=1..3</t>
   </si>
   <si>
-    <t>AALoadoutRecords</t>
-  </si>
-  <si>
-    <t>ca818c3e9587d3f0</t>
-  </si>
-  <si>
-    <t>AAProgressRecords</t>
-  </si>
-  <si>
-    <t>d1dcd76b7da2d723</t>
-  </si>
-  <si>
-    <t>AAKingStates</t>
-  </si>
-  <si>
-    <t>6eb8618cc70e8adb</t>
+    <t>ArbLoadoutRecords</t>
+  </si>
+  <si>
+    <t>8f962f87d981d726</t>
+  </si>
+  <si>
+    <t>ArbProgressRecords</t>
+  </si>
+  <si>
+    <t>841d6697256ce8d5</t>
+  </si>
+  <si>
+    <t>ArbKingStates</t>
+  </si>
+  <si>
+    <t>05b940e2f1ce7343</t>
   </si>
   <si>
     <t>range=1..1000</t>
   </si>
   <si>
-    <t>AAKingProtection</t>
-  </si>
-  <si>
-    <t>76e01b96f0266e66</t>
-  </si>
-  <si>
-    <t>AAClocks</t>
-  </si>
-  <si>
-    <t>6fae731299790b03</t>
+    <t>ArbKingProtection</t>
+  </si>
+  <si>
+    <t>500af8a16426580c</t>
+  </si>
+  <si>
+    <t>ArbClocks</t>
+  </si>
+  <si>
+    <t>72845d73c8f623db</t>
   </si>
   <si>
     <t>stage_stable_keys</t>
@@ -302,19 +302,19 @@
     <t>parser=split;separator=|;length=0..5</t>
   </si>
   <si>
-    <t>AAQuadrantOptions</t>
-  </si>
-  <si>
-    <t>aa248a8db4b193fe</t>
+    <t>ArbQuadrantOptions</t>
+  </si>
+  <si>
+    <t>6445cff54a147672</t>
   </si>
   <si>
     <t>source_numeric_id</t>
   </si>
   <si>
-    <t>AAQuadrantSelections</t>
-  </si>
-  <si>
-    <t>faad7d6eee209870</t>
+    <t>ArbQuadrantSelections</t>
+  </si>
+  <si>
+    <t>3894955cac865078</t>
   </si>
   <si>
     <t>option_stable_keys</t>
@@ -323,16 +323,16 @@
     <t>parser=split;separator=|;length=0..3</t>
   </si>
   <si>
-    <t>AATargets</t>
-  </si>
-  <si>
-    <t>cea580f3083e97b6</t>
-  </si>
-  <si>
-    <t>AAObjectives</t>
-  </si>
-  <si>
-    <t>6d2e276da7738fdd</t>
+    <t>ArbTargets</t>
+  </si>
+  <si>
+    <t>f5e1a193a88bfe9a</t>
+  </si>
+  <si>
+    <t>ArbObjectives</t>
+  </si>
+  <si>
+    <t>99b25f3f6c72a26f</t>
   </si>
   <si>
     <t>target_stable_keys</t>
@@ -341,16 +341,16 @@
     <t>parser=split;separator=|;length=0..7</t>
   </si>
   <si>
-    <t>AAStageResults</t>
-  </si>
-  <si>
-    <t>d03cc1d19afbb12b</t>
-  </si>
-  <si>
-    <t>AAAggregations</t>
-  </si>
-  <si>
-    <t>331f358e56d29983</t>
+    <t>ArbStageResults</t>
+  </si>
+  <si>
+    <t>945c2e477edd7b17</t>
+  </si>
+  <si>
+    <t>ArbAggregations</t>
+  </si>
+  <si>
+    <t>c7c85c9f284a79df</t>
   </si>
 </sst>
 </file>
@@ -773,10 +773,10 @@
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="7" width="12.7109375" style="5" customWidth="1"/>
     <col min="8" max="8" width="13.7109375" style="5" customWidth="1"/>
-    <col min="9" max="9" width="17.7109375" style="5" customWidth="1"/>
-    <col min="10" max="10" width="21.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="23.7109375" style="5" customWidth="1"/>
-    <col min="12" max="12" width="24.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="18.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="22.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="24.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="25.7109375" style="5" customWidth="1"/>
     <col min="13" max="13" width="19.7109375" style="5" customWidth="1"/>
     <col min="14" max="14" width="14.7109375" style="5" customWidth="1"/>
     <col min="15" max="16" width="12.7109375" style="5" customWidth="1"/>
@@ -1097,16 +1097,16 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AA, Shared" promptTitle="AAOwnership enum" prompt="Select a value from the dropdown." sqref="I8:I1007">
-      <formula1>"AA,Shared"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="AACoverageState enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AnomalyArbitration, Shared" promptTitle="ArbOwnership enum" prompt="Select a value from the dropdown." sqref="I8:I1007">
+      <formula1>"AnomalyArbitration,Shared"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="ArbCoverageState enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="AAEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="ArbEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="AAMechanismQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="ArbMechanismQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
       <formula1>"ExactProgram,ExactRelationship,ObservedBehavior,IdentityCrossCheck,PolicyBoundary,ContextOnly"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid boolean value" error="Value must be true or false." promptTitle="Boolean" prompt="Select true or false." sqref="Q8:Q1007">
@@ -1124,13 +1124,13 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" style="5" customWidth="1"/>
     <col min="4" max="8" width="12.7109375" style="5" customWidth="1"/>
     <col min="9" max="9" width="13.7109375" style="5" customWidth="1"/>
-    <col min="10" max="10" width="17.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="21.7109375" style="5" customWidth="1"/>
-    <col min="12" max="12" width="23.7109375" style="5" customWidth="1"/>
-    <col min="13" max="13" width="24.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="18.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="22.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="24.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="25.7109375" style="5" customWidth="1"/>
     <col min="14" max="14" width="19.7109375" style="5" customWidth="1"/>
     <col min="15" max="15" width="14.7109375" style="5" customWidth="1"/>
     <col min="16" max="16" width="12.7109375" style="5" customWidth="1"/>
@@ -1453,16 +1453,16 @@
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AA, Shared" promptTitle="AAOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"AA,Shared"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="AACoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AnomalyArbitration, Shared" promptTitle="ArbOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"AnomalyArbitration,Shared"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="ArbCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="AAEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="ArbEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
       <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="AAMechanismQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="ArbMechanismQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
       <formula1>"ExactProgram,ExactRelationship,ObservedBehavior,IdentityCrossCheck,PolicyBoundary,ContextOnly"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid boolean value" error="Value must be true or false." promptTitle="Boolean" prompt="Select true or false." sqref="Q8:Q1007">
@@ -1480,15 +1480,15 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" style="5" customWidth="1"/>
     <col min="4" max="5" width="12.7109375" style="5" customWidth="1"/>
     <col min="6" max="6" width="17.7109375" style="5" customWidth="1"/>
     <col min="7" max="9" width="12.7109375" style="5" customWidth="1"/>
     <col min="10" max="10" width="13.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="17.7109375" style="5" customWidth="1"/>
-    <col min="12" max="12" width="21.7109375" style="5" customWidth="1"/>
-    <col min="13" max="13" width="23.7109375" style="5" customWidth="1"/>
-    <col min="14" max="14" width="24.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="18.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="24.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="25.7109375" style="5" customWidth="1"/>
     <col min="15" max="15" width="19.7109375" style="5" customWidth="1"/>
     <col min="16" max="16" width="14.7109375" style="5" customWidth="1"/>
     <col min="17" max="17" width="12.7109375" style="5" customWidth="1"/>
@@ -1827,16 +1827,16 @@
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AA, Shared" promptTitle="AAOwnership enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
-      <formula1>"AA,Shared"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="AACoverageState enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AnomalyArbitration, Shared" promptTitle="ArbOwnership enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+      <formula1>"AnomalyArbitration,Shared"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="ArbCoverageState enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="AAEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="ArbEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
       <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="AAMechanismQuality enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="ArbMechanismQuality enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
       <formula1>"ExactProgram,ExactRelationship,ObservedBehavior,IdentityCrossCheck,PolicyBoundary,ContextOnly"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid boolean value" error="Value must be true or false." promptTitle="Boolean" prompt="Select true or false." sqref="R8:R1007">
@@ -1854,15 +1854,15 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" style="5" customWidth="1"/>
     <col min="4" max="4" width="12.7109375" style="5" customWidth="1"/>
     <col min="5" max="5" width="17.7109375" style="5" customWidth="1"/>
     <col min="6" max="9" width="12.7109375" style="5" customWidth="1"/>
     <col min="10" max="10" width="13.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="17.7109375" style="5" customWidth="1"/>
-    <col min="12" max="12" width="21.7109375" style="5" customWidth="1"/>
-    <col min="13" max="13" width="23.7109375" style="5" customWidth="1"/>
-    <col min="14" max="14" width="24.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="18.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="24.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="25.7109375" style="5" customWidth="1"/>
     <col min="15" max="15" width="19.7109375" style="5" customWidth="1"/>
     <col min="16" max="16" width="14.7109375" style="5" customWidth="1"/>
     <col min="17" max="17" width="12.7109375" style="5" customWidth="1"/>
@@ -2201,16 +2201,16 @@
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AA, Shared" promptTitle="AAOwnership enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
-      <formula1>"AA,Shared"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="AACoverageState enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AnomalyArbitration, Shared" promptTitle="ArbOwnership enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+      <formula1>"AnomalyArbitration,Shared"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="ArbCoverageState enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="AAEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="ArbEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
       <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="AAMechanismQuality enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="ArbMechanismQuality enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
       <formula1>"ExactProgram,ExactRelationship,ObservedBehavior,IdentityCrossCheck,PolicyBoundary,ContextOnly"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid boolean value" error="Value must be true or false." promptTitle="Boolean" prompt="Select true or false." sqref="R8:R1007">
@@ -2228,15 +2228,15 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" style="5" customWidth="1"/>
     <col min="4" max="5" width="12.7109375" style="5" customWidth="1"/>
     <col min="6" max="6" width="18.7109375" style="5" customWidth="1"/>
     <col min="7" max="9" width="12.7109375" style="5" customWidth="1"/>
     <col min="10" max="10" width="13.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="17.7109375" style="5" customWidth="1"/>
-    <col min="12" max="12" width="21.7109375" style="5" customWidth="1"/>
-    <col min="13" max="13" width="23.7109375" style="5" customWidth="1"/>
-    <col min="14" max="14" width="24.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="18.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="24.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="25.7109375" style="5" customWidth="1"/>
     <col min="15" max="15" width="19.7109375" style="5" customWidth="1"/>
     <col min="16" max="16" width="14.7109375" style="5" customWidth="1"/>
     <col min="17" max="17" width="12.7109375" style="5" customWidth="1"/>
@@ -2575,16 +2575,16 @@
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AA, Shared" promptTitle="AAOwnership enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
-      <formula1>"AA,Shared"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="AACoverageState enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AnomalyArbitration, Shared" promptTitle="ArbOwnership enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+      <formula1>"AnomalyArbitration,Shared"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="ArbCoverageState enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="AAEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="ArbEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
       <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="AAMechanismQuality enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="ArbMechanismQuality enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
       <formula1>"ExactProgram,ExactRelationship,ObservedBehavior,IdentityCrossCheck,PolicyBoundary,ContextOnly"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid boolean value" error="Value must be true or false." promptTitle="Boolean" prompt="Select true or false." sqref="R8:R1007">
@@ -2602,15 +2602,15 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" style="5" customWidth="1"/>
     <col min="4" max="4" width="12.7109375" style="5" customWidth="1"/>
     <col min="5" max="5" width="17.7109375" style="5" customWidth="1"/>
     <col min="6" max="9" width="12.7109375" style="5" customWidth="1"/>
     <col min="10" max="10" width="13.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="17.7109375" style="5" customWidth="1"/>
-    <col min="12" max="12" width="21.7109375" style="5" customWidth="1"/>
-    <col min="13" max="13" width="23.7109375" style="5" customWidth="1"/>
-    <col min="14" max="14" width="24.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="18.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="24.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="25.7109375" style="5" customWidth="1"/>
     <col min="15" max="15" width="19.7109375" style="5" customWidth="1"/>
     <col min="16" max="16" width="14.7109375" style="5" customWidth="1"/>
     <col min="17" max="17" width="12.7109375" style="5" customWidth="1"/>
@@ -2949,16 +2949,16 @@
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AA, Shared" promptTitle="AAOwnership enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
-      <formula1>"AA,Shared"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="AACoverageState enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AnomalyArbitration, Shared" promptTitle="ArbOwnership enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+      <formula1>"AnomalyArbitration,Shared"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="ArbCoverageState enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="AAEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="ArbEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
       <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="AAMechanismQuality enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="ArbMechanismQuality enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
       <formula1>"ExactProgram,ExactRelationship,ObservedBehavior,IdentityCrossCheck,PolicyBoundary,ContextOnly"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid boolean value" error="Value must be true or false." promptTitle="Boolean" prompt="Select true or false." sqref="R8:R1007">
@@ -2976,15 +2976,15 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" style="5" customWidth="1"/>
     <col min="4" max="5" width="12.7109375" style="5" customWidth="1"/>
     <col min="6" max="6" width="18.7109375" style="5" customWidth="1"/>
     <col min="7" max="9" width="12.7109375" style="5" customWidth="1"/>
     <col min="10" max="10" width="13.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="17.7109375" style="5" customWidth="1"/>
-    <col min="12" max="12" width="21.7109375" style="5" customWidth="1"/>
-    <col min="13" max="13" width="23.7109375" style="5" customWidth="1"/>
-    <col min="14" max="14" width="24.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="18.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="24.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="25.7109375" style="5" customWidth="1"/>
     <col min="15" max="15" width="19.7109375" style="5" customWidth="1"/>
     <col min="16" max="16" width="14.7109375" style="5" customWidth="1"/>
     <col min="17" max="17" width="12.7109375" style="5" customWidth="1"/>
@@ -3323,16 +3323,16 @@
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AA, Shared" promptTitle="AAOwnership enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
-      <formula1>"AA,Shared"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="AACoverageState enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AnomalyArbitration, Shared" promptTitle="ArbOwnership enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+      <formula1>"AnomalyArbitration,Shared"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="ArbCoverageState enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="AAEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="ArbEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
       <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="AAMechanismQuality enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="ArbMechanismQuality enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
       <formula1>"ExactProgram,ExactRelationship,ObservedBehavior,IdentityCrossCheck,PolicyBoundary,ContextOnly"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid boolean value" error="Value must be true or false." promptTitle="Boolean" prompt="Select true or false." sqref="R8:R1007">
@@ -3350,15 +3350,15 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" style="5" customWidth="1"/>
     <col min="4" max="5" width="12.7109375" style="5" customWidth="1"/>
     <col min="6" max="6" width="18.7109375" style="5" customWidth="1"/>
     <col min="7" max="9" width="12.7109375" style="5" customWidth="1"/>
     <col min="10" max="10" width="13.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="17.7109375" style="5" customWidth="1"/>
-    <col min="12" max="12" width="21.7109375" style="5" customWidth="1"/>
-    <col min="13" max="13" width="23.7109375" style="5" customWidth="1"/>
-    <col min="14" max="14" width="24.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="18.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="24.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="25.7109375" style="5" customWidth="1"/>
     <col min="15" max="15" width="19.7109375" style="5" customWidth="1"/>
     <col min="16" max="16" width="14.7109375" style="5" customWidth="1"/>
     <col min="17" max="17" width="12.7109375" style="5" customWidth="1"/>
@@ -3697,16 +3697,16 @@
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AA, Shared" promptTitle="AAOwnership enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
-      <formula1>"AA,Shared"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="AACoverageState enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AnomalyArbitration, Shared" promptTitle="ArbOwnership enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+      <formula1>"AnomalyArbitration,Shared"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="ArbCoverageState enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="AAEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="ArbEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
       <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="AAMechanismQuality enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="ArbMechanismQuality enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
       <formula1>"ExactProgram,ExactRelationship,ObservedBehavior,IdentityCrossCheck,PolicyBoundary,ContextOnly"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid boolean value" error="Value must be true or false." promptTitle="Boolean" prompt="Select true or false." sqref="R8:R1007">
@@ -3724,15 +3724,15 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" style="5" customWidth="1"/>
     <col min="4" max="5" width="12.7109375" style="5" customWidth="1"/>
     <col min="6" max="6" width="17.7109375" style="5" customWidth="1"/>
     <col min="7" max="9" width="12.7109375" style="5" customWidth="1"/>
     <col min="10" max="10" width="13.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="17.7109375" style="5" customWidth="1"/>
-    <col min="12" max="12" width="21.7109375" style="5" customWidth="1"/>
-    <col min="13" max="13" width="23.7109375" style="5" customWidth="1"/>
-    <col min="14" max="14" width="24.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="18.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="24.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="25.7109375" style="5" customWidth="1"/>
     <col min="15" max="15" width="19.7109375" style="5" customWidth="1"/>
     <col min="16" max="16" width="14.7109375" style="5" customWidth="1"/>
     <col min="17" max="17" width="12.7109375" style="5" customWidth="1"/>
@@ -4071,16 +4071,16 @@
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AA, Shared" promptTitle="AAOwnership enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
-      <formula1>"AA,Shared"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="AACoverageState enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AnomalyArbitration, Shared" promptTitle="ArbOwnership enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+      <formula1>"AnomalyArbitration,Shared"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="ArbCoverageState enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="AAEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="ArbEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
       <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="AAMechanismQuality enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="ArbMechanismQuality enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
       <formula1>"ExactProgram,ExactRelationship,ObservedBehavior,IdentityCrossCheck,PolicyBoundary,ContextOnly"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid boolean value" error="Value must be true or false." promptTitle="Boolean" prompt="Select true or false." sqref="R8:R1007">
@@ -4098,15 +4098,15 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" style="5" customWidth="1"/>
     <col min="4" max="4" width="12.7109375" style="5" customWidth="1"/>
     <col min="5" max="5" width="15.7109375" style="5" customWidth="1"/>
     <col min="6" max="8" width="12.7109375" style="5" customWidth="1"/>
     <col min="9" max="9" width="13.7109375" style="5" customWidth="1"/>
-    <col min="10" max="10" width="17.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="21.7109375" style="5" customWidth="1"/>
-    <col min="12" max="12" width="23.7109375" style="5" customWidth="1"/>
-    <col min="13" max="13" width="24.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="18.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="22.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="24.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="25.7109375" style="5" customWidth="1"/>
     <col min="14" max="14" width="19.7109375" style="5" customWidth="1"/>
     <col min="15" max="15" width="14.7109375" style="5" customWidth="1"/>
     <col min="16" max="17" width="12.7109375" style="5" customWidth="1"/>
@@ -4441,16 +4441,16 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AA, Shared" promptTitle="AAOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"AA,Shared"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="AACoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AnomalyArbitration, Shared" promptTitle="ArbOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"AnomalyArbitration,Shared"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="ArbCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="AAEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="ArbEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
       <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="AAMechanismQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="ArbMechanismQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
       <formula1>"ExactProgram,ExactRelationship,ObservedBehavior,IdentityCrossCheck,PolicyBoundary,ContextOnly"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid boolean value" error="Value must be true or false." promptTitle="Boolean" prompt="Select true or false." sqref="R8:R1007">
@@ -4468,18 +4468,18 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="5" customWidth="1"/>
     <col min="4" max="4" width="12.7109375" style="5" customWidth="1"/>
     <col min="5" max="5" width="15.7109375" style="5" customWidth="1"/>
     <col min="6" max="6" width="12.7109375" style="5" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" style="5" customWidth="1"/>
-    <col min="8" max="8" width="18.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="18.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="19.7109375" style="5" customWidth="1"/>
     <col min="9" max="11" width="12.7109375" style="5" customWidth="1"/>
     <col min="12" max="12" width="13.7109375" style="5" customWidth="1"/>
-    <col min="13" max="13" width="17.7109375" style="5" customWidth="1"/>
-    <col min="14" max="14" width="21.7109375" style="5" customWidth="1"/>
-    <col min="15" max="15" width="23.7109375" style="5" customWidth="1"/>
-    <col min="16" max="16" width="24.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="18.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="22.7109375" style="5" customWidth="1"/>
+    <col min="15" max="15" width="24.7109375" style="5" customWidth="1"/>
+    <col min="16" max="16" width="25.7109375" style="5" customWidth="1"/>
     <col min="17" max="17" width="19.7109375" style="5" customWidth="1"/>
     <col min="18" max="18" width="14.7109375" style="5" customWidth="1"/>
     <col min="19" max="20" width="12.7109375" style="5" customWidth="1"/>
@@ -4862,22 +4862,22 @@
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Knight, King" promptTitle="AAStageKind enum" prompt="Select a value from the dropdown." sqref="G8:G1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Knight, King" promptTitle="ArbStageKind enum" prompt="Select a value from the dropdown." sqref="G8:G1007">
       <formula1>"Knight,King"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Normal, Plight" promptTitle="AADifficulty enum" prompt="Select a value from the dropdown." sqref="H8:H1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Normal, Plight" promptTitle="ArbDifficulty enum" prompt="Select a value from the dropdown." sqref="H8:H1007">
       <formula1>"Normal,Plight"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AA, Shared" promptTitle="AAOwnership enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
-      <formula1>"AA,Shared"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="AACoverageState enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AnomalyArbitration, Shared" promptTitle="ArbOwnership enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+      <formula1>"AnomalyArbitration,Shared"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="ArbCoverageState enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="AAEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="O8:O1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="ArbEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="O8:O1007">
       <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="AAMechanismQuality enum" prompt="Select a value from the dropdown." sqref="P8:P1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="ArbMechanismQuality enum" prompt="Select a value from the dropdown." sqref="P8:P1007">
       <formula1>"ExactProgram,ExactRelationship,ObservedBehavior,IdentityCrossCheck,PolicyBoundary,ContextOnly"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid boolean value" error="Value must be true or false." promptTitle="Boolean" prompt="Select true or false." sqref="U8:U1007">
@@ -4895,13 +4895,13 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" style="5" customWidth="1"/>
     <col min="4" max="7" width="12.7109375" style="5" customWidth="1"/>
     <col min="8" max="8" width="13.7109375" style="5" customWidth="1"/>
-    <col min="9" max="9" width="17.7109375" style="5" customWidth="1"/>
-    <col min="10" max="10" width="21.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="23.7109375" style="5" customWidth="1"/>
-    <col min="12" max="12" width="24.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="18.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="22.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="24.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="25.7109375" style="5" customWidth="1"/>
     <col min="13" max="13" width="19.7109375" style="5" customWidth="1"/>
     <col min="14" max="14" width="14.7109375" style="5" customWidth="1"/>
     <col min="15" max="16" width="12.7109375" style="5" customWidth="1"/>
@@ -5220,16 +5220,16 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AA, Shared" promptTitle="AAOwnership enum" prompt="Select a value from the dropdown." sqref="I8:I1007">
-      <formula1>"AA,Shared"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="AACoverageState enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AnomalyArbitration, Shared" promptTitle="ArbOwnership enum" prompt="Select a value from the dropdown." sqref="I8:I1007">
+      <formula1>"AnomalyArbitration,Shared"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="ArbCoverageState enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="AAEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="ArbEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="AAMechanismQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="ArbMechanismQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
       <formula1>"ExactProgram,ExactRelationship,ObservedBehavior,IdentityCrossCheck,PolicyBoundary,ContextOnly"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid boolean value" error="Value must be true or false." promptTitle="Boolean" prompt="Select true or false." sqref="Q8:Q1007">
@@ -5247,13 +5247,13 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" style="5" customWidth="1"/>
     <col min="4" max="8" width="12.7109375" style="5" customWidth="1"/>
     <col min="9" max="9" width="13.7109375" style="5" customWidth="1"/>
-    <col min="10" max="10" width="17.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="21.7109375" style="5" customWidth="1"/>
-    <col min="12" max="12" width="23.7109375" style="5" customWidth="1"/>
-    <col min="13" max="13" width="24.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="18.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="22.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="24.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="25.7109375" style="5" customWidth="1"/>
     <col min="14" max="14" width="19.7109375" style="5" customWidth="1"/>
     <col min="15" max="15" width="14.7109375" style="5" customWidth="1"/>
     <col min="16" max="17" width="12.7109375" style="5" customWidth="1"/>
@@ -5592,16 +5592,16 @@
       <formula1>1</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AA, Shared" promptTitle="AAOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"AA,Shared"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="AACoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AnomalyArbitration, Shared" promptTitle="ArbOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"AnomalyArbitration,Shared"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="ArbCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="AAEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="ArbEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
       <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="AAMechanismQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="ArbMechanismQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
       <formula1>"ExactProgram,ExactRelationship,ObservedBehavior,IdentityCrossCheck,PolicyBoundary,ContextOnly"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid boolean value" error="Value must be true or false." promptTitle="Boolean" prompt="Select true or false." sqref="R8:R1007">
@@ -5619,14 +5619,14 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="5" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" style="5" customWidth="1"/>
     <col min="5" max="9" width="12.7109375" style="5" customWidth="1"/>
     <col min="10" max="10" width="13.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="17.7109375" style="5" customWidth="1"/>
-    <col min="12" max="12" width="21.7109375" style="5" customWidth="1"/>
-    <col min="13" max="13" width="23.7109375" style="5" customWidth="1"/>
-    <col min="14" max="14" width="24.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="18.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="24.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="25.7109375" style="5" customWidth="1"/>
     <col min="15" max="15" width="19.7109375" style="5" customWidth="1"/>
     <col min="16" max="16" width="14.7109375" style="5" customWidth="1"/>
     <col min="17" max="18" width="12.7109375" style="5" customWidth="1"/>
@@ -5979,16 +5979,16 @@
       <formula1>1</formula1>
       <formula2>3</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AA, Shared" promptTitle="AAOwnership enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
-      <formula1>"AA,Shared"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="AACoverageState enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AnomalyArbitration, Shared" promptTitle="ArbOwnership enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+      <formula1>"AnomalyArbitration,Shared"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="ArbCoverageState enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="AAEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="ArbEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
       <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="AAMechanismQuality enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="ArbMechanismQuality enum" prompt="Select a value from the dropdown." sqref="N8:N1007">
       <formula1>"ExactProgram,ExactRelationship,ObservedBehavior,IdentityCrossCheck,PolicyBoundary,ContextOnly"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid boolean value" error="Value must be true or false." promptTitle="Boolean" prompt="Select true or false." sqref="S8:S1007">
@@ -6006,13 +6006,13 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" style="5" customWidth="1"/>
     <col min="4" max="8" width="12.7109375" style="5" customWidth="1"/>
     <col min="9" max="9" width="13.7109375" style="5" customWidth="1"/>
-    <col min="10" max="10" width="17.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="21.7109375" style="5" customWidth="1"/>
-    <col min="12" max="12" width="23.7109375" style="5" customWidth="1"/>
-    <col min="13" max="13" width="24.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="18.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="22.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="24.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="25.7109375" style="5" customWidth="1"/>
     <col min="14" max="14" width="19.7109375" style="5" customWidth="1"/>
     <col min="15" max="15" width="14.7109375" style="5" customWidth="1"/>
     <col min="16" max="17" width="12.7109375" style="5" customWidth="1"/>
@@ -6351,16 +6351,16 @@
       <formula1>1</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AA, Shared" promptTitle="AAOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"AA,Shared"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="AACoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AnomalyArbitration, Shared" promptTitle="ArbOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"AnomalyArbitration,Shared"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="ArbCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="AAEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="ArbEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
       <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="AAMechanismQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="ArbMechanismQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
       <formula1>"ExactProgram,ExactRelationship,ObservedBehavior,IdentityCrossCheck,PolicyBoundary,ContextOnly"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid boolean value" error="Value must be true or false." promptTitle="Boolean" prompt="Select true or false." sqref="R8:R1007">
@@ -6378,13 +6378,13 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" style="5" customWidth="1"/>
     <col min="4" max="8" width="12.7109375" style="5" customWidth="1"/>
     <col min="9" max="9" width="13.7109375" style="5" customWidth="1"/>
-    <col min="10" max="10" width="17.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="21.7109375" style="5" customWidth="1"/>
-    <col min="12" max="12" width="23.7109375" style="5" customWidth="1"/>
-    <col min="13" max="13" width="24.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="18.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="22.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="24.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="25.7109375" style="5" customWidth="1"/>
     <col min="14" max="14" width="19.7109375" style="5" customWidth="1"/>
     <col min="15" max="15" width="14.7109375" style="5" customWidth="1"/>
     <col min="16" max="17" width="12.7109375" style="5" customWidth="1"/>
@@ -6723,16 +6723,16 @@
       <formula1>1</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AA, Shared" promptTitle="AAOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"AA,Shared"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="AACoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AnomalyArbitration, Shared" promptTitle="ArbOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"AnomalyArbitration,Shared"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="ArbCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="AAEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="ArbEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
       <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="AAMechanismQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="ArbMechanismQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
       <formula1>"ExactProgram,ExactRelationship,ObservedBehavior,IdentityCrossCheck,PolicyBoundary,ContextOnly"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid boolean value" error="Value must be true or false." promptTitle="Boolean" prompt="Select true or false." sqref="R8:R1007">
@@ -6750,13 +6750,13 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" style="5" customWidth="1"/>
     <col min="4" max="8" width="12.7109375" style="5" customWidth="1"/>
     <col min="9" max="9" width="13.7109375" style="5" customWidth="1"/>
-    <col min="10" max="10" width="17.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="21.7109375" style="5" customWidth="1"/>
-    <col min="12" max="12" width="23.7109375" style="5" customWidth="1"/>
-    <col min="13" max="13" width="24.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="18.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="22.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="24.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="25.7109375" style="5" customWidth="1"/>
     <col min="14" max="14" width="19.7109375" style="5" customWidth="1"/>
     <col min="15" max="15" width="14.7109375" style="5" customWidth="1"/>
     <col min="16" max="16" width="12.7109375" style="5" customWidth="1"/>
@@ -7079,16 +7079,16 @@
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AA, Shared" promptTitle="AAOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"AA,Shared"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="AACoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: AnomalyArbitration, Shared" promptTitle="ArbOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"AnomalyArbitration,Shared"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked" promptTitle="ArbCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="AAEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="ArbEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
       <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="AAMechanismQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactProgram, ExactRelationship, ObservedBehavior, IdentityCrossCheck, PolicyBoundary, ContextOnly" promptTitle="ArbMechanismQuality enum" prompt="Select a value from the dropdown." sqref="M8:M1007">
       <formula1>"ExactProgram,ExactRelationship,ObservedBehavior,IdentityCrossCheck,PolicyBoundary,ContextOnly"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid boolean value" error="Value must be true or false." promptTitle="Boolean" prompt="Select true or false." sqref="Q8:Q1007">

</xml_diff>